<commit_message>
Update route model: Marijampolė route, bridge sale sheet, team info
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EQQBp74E19JPxXkooia4GN
</commit_message>
<xml_diff>
--- a/klaipeda-h2/Klaipeda_H2_Route_Model.xlsx
+++ b/klaipeda-h2/Klaipeda_H2_Route_Model.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Inputs" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Routes" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Capacity" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Sensitivity" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Bridge Sale" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Sensitivity" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="134">
-  <si>
-    <t xml:space="preserve">Klaipėda Port green hydrogen – freight route model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portathon 2026 · Challenge 1: the most efficient hydrogen freight route in the EU</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="167">
+  <si>
+    <t xml:space="preserve">Baltic H₂ Gateway – Klaipėda green hydrogen route model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUVIA Team · Klaipėdos valstybinė kolegija · Portathon 2026, Port of Klaipėda Challenge 1</t>
   </si>
   <si>
     <t xml:space="preserve">What this does</t>
@@ -44,7 +45,7 @@
     <t xml:space="preserve">1. Change the yellow cells on the Inputs sheet (hydrogen price, diesel price, CO₂ price, trucks per route).</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Read the results on Routes (per truck), Capacity (whole plan) and Sensitivity (price × CO₂ grid).</t>
+    <t xml:space="preserve">2. Read the results on Routes (per truck), Capacity (whole plan), Bridge Sale (1.5 t trial) and Sensitivity (price × CO₂ grid).</t>
   </si>
   <si>
     <t xml:space="preserve">3. Everything else is a formula – do not overwrite it.</t>
@@ -86,6 +87,9 @@
     <t xml:space="preserve">€200/t CO₂ scenario and €8–30/kg price points: team's own workshop notes</t>
   </si>
   <si>
+    <t xml:space="preserve">Team: Mahyi Eddine Bouaffar, Chukwuemeka Onyemejor, Mokhtar Ounis, Salah Djoudi, Lotfi Boumaza · Mentor: Lina Gelažnikienė</t>
+  </si>
+  <si>
     <t xml:space="preserve">Inputs – change the blue numbers</t>
   </si>
   <si>
@@ -332,6 +336,12 @@
     <t xml:space="preserve">Klaipėda ↔ Riga (Riga station not green today)</t>
   </si>
   <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klaipėda ↔ Marijampolė via Kaunas (Via Baltica; refuel at the planned Marijampolė 700-bar station)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
@@ -341,7 +351,7 @@
     <t xml:space="preserve">Route A: 6 short round trips a day (~180 km) for a truck moving containers between the port and nearby sites.</t>
   </si>
   <si>
-    <t xml:space="preserve">'Fits one fill?' checks one round trip against the tank minus the safety reserve. Route C/D/E need a refuel at the far end.</t>
+    <t xml:space="preserve">'Fits one fill?' checks one round trip against the tank minus the safety reserve. Routes C–F need a refuel at the far end.</t>
   </si>
   <si>
     <t xml:space="preserve">Extra cost per truck per year includes the truck cost premium from Inputs (0 until you add a quote).</t>
@@ -350,6 +360,9 @@
     <t xml:space="preserve">CO₂ saved is tank-to-wheel for diesel replaced by green hydrogen.</t>
   </si>
   <si>
+    <t xml:space="preserve">Route F becomes possible once the Marijampolė station opens (Baltic H₂ Gateway stage 3, 2028+); it links Lithuania to Poland on Via Baltica.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Does the plan fit the plant? – supply vs demand</t>
   </si>
   <si>
@@ -411,6 +424,93 @@
   </si>
   <si>
     <t xml:space="preserve">Pilot volume to ask for (Routes A + B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bridge sale – 1.5 t trial batch to industry (deck stage 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue = inputs. Delivered by 350-bar tube trailer; no new vehicles needed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trial batch size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deck stage 1: 1.5 t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price – low case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Benchmark: €8/kg truck H₂ in Germany (2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price – high case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upper benchmark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue – low case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue – high case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of sellable hydrogen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trial vs what the port can sell in a year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days of spare output used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">working days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How long the plant needs to make the batch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Candidate buyers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Road km from Klaipėda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use of hydrogen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orlen Lietuva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mažeikiai refinery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hydrotreating – removing sulphur from diesel and petrol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Achema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jonava fertiliser plant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feedstock for ammonia (NH₃) – replacing grey hydrogen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distances are approximate road km. Final price depends on buyer terms, purity and delivery.</t>
   </si>
   <si>
     <t xml:space="preserve">Extra cost of hydrogen vs diesel, € per km – hydrogen price × CO₂ price</t>
@@ -432,7 +532,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.0%;\(0.0%\);\-"/>
@@ -440,8 +540,13 @@
     <numFmt numFmtId="168" formatCode="\€#,##0;&quot;(€&quot;#,##0\);\-"/>
     <numFmt numFmtId="169" formatCode="0.00"/>
     <numFmt numFmtId="170" formatCode="#,##0.0;\(#,##0.0\);\-"/>
+    <numFmt numFmtId="171" formatCode="#,##0;\(#,##0\);\-"/>
+    <numFmt numFmtId="172" formatCode="\€0.00"/>
+    <numFmt numFmtId="173" formatCode="\€#,##0;&quot;(€&quot;#,##0\);\-"/>
+    <numFmt numFmtId="174" formatCode="0.0%"/>
+    <numFmt numFmtId="175" formatCode="0.0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -541,9 +646,67 @@
       <charset val="1"/>
     </font>
     <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color rgb="FF555555"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF555555"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -624,16 +787,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="57">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -645,47 +812,51 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -733,55 +904,115 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1037,122 +1268,127 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="130"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="130"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1174,276 +1410,276 @@
   <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="90"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="5" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="C4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="D4" s="7" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="6" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="B5" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="9" t="n">
         <v>127000</v>
       </c>
-      <c r="D5" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="6" t="s">
+      <c r="E5" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="7" t="n">
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="9" t="n">
         <v>500</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" s="9" t="s">
+      <c r="D6" s="10" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="6" t="s">
+      <c r="E6" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="10" t="n">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="E7" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="6" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="B8" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="9" t="s">
+      <c r="D8" s="10" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="6" t="s">
+      <c r="E8" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="11" t="n">
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="13" t="n">
         <v>1.2</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="E9" s="9" t="s">
+      <c r="D9" s="10" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="6" t="s">
+      <c r="E9" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="12" t="n">
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="9" t="s">
+      <c r="D10" s="10" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="6" t="s">
+      <c r="E10" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="13" t="n">
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="15" t="n">
         <v>2.65</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" s="9" t="s">
+      <c r="D11" s="10" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="E11" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="6" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="B12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="16" t="n">
         <v>31.5</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E12" s="9" t="s">
+      <c r="D12" s="10" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B13" s="6" t="s">
+      <c r="E12" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="14" t="n">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="16" t="n">
         <v>7.5</v>
       </c>
-      <c r="D13" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" s="9" t="s">
+      <c r="D13" s="10" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B14" s="6" t="s">
+      <c r="E13" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="14" t="n">
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="D14" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B15" s="6" t="s">
+      <c r="E14" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="10" t="n">
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="12" t="n">
         <v>0.15</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B16" s="6" t="s">
+      <c r="D15" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="7" t="n">
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="9" t="n">
         <v>250</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="E16" s="9" t="s">
+      <c r="D16" s="10" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B17" s="6" t="s">
+      <c r="E16" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="12" t="n">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="E17" s="9" t="s">
+      <c r="D17" s="10" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B18" s="6" t="s">
+      <c r="E17" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C18" s="15" t="n">
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="E18" s="9" t="s">
+      <c r="D18" s="10" t="s">
         <v>70</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1462,488 +1698,569 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:S18"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>72</v>
       </c>
     </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="A4" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="C4" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="D4" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="E4" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="G4" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="H4" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="I4" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="J4" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="K4" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="L4" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="M4" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="O4" s="5" t="s">
+      <c r="N4" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="P4" s="5" t="s">
+      <c r="O4" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="Q4" s="5" t="s">
+      <c r="P4" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="R4" s="5" t="s">
+      <c r="Q4" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="S4" s="5" t="s">
+      <c r="R4" s="7" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
+      <c r="S4" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="17" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="B5" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="D5" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="20" t="n">
+      <c r="F5" s="22" t="n">
         <f aca="false">2*C5*D5</f>
         <v>180</v>
       </c>
-      <c r="G5" s="21" t="n">
+      <c r="G5" s="23" t="n">
         <f aca="false">F5*Inputs!$C$13/100</f>
         <v>13.5</v>
       </c>
-      <c r="H5" s="22" t="n">
+      <c r="H5" s="24" t="n">
         <f aca="false">Inputs!$C$12*(1-Inputs!$C$15)</f>
         <v>26.775</v>
       </c>
-      <c r="I5" s="23" t="str">
+      <c r="I5" s="25" t="str">
         <f aca="false">IF(G5/D5&lt;=H5,"Yes","No – refuel at far end")</f>
         <v>Yes</v>
       </c>
-      <c r="J5" s="20" t="n">
+      <c r="J5" s="22" t="n">
         <f aca="false">G5*Inputs!$C$16</f>
         <v>3375</v>
       </c>
-      <c r="K5" s="24" t="n">
+      <c r="K5" s="26" t="n">
         <f aca="false">Inputs!$C$14/100*Inputs!$C$9</f>
         <v>0.36</v>
       </c>
-      <c r="L5" s="25" t="n">
+      <c r="L5" s="27" t="n">
         <f aca="false">Inputs!$C$14/100*Inputs!$C$11/1000*Inputs!$C$10</f>
         <v>0</v>
       </c>
-      <c r="M5" s="24" t="n">
+      <c r="M5" s="26" t="n">
         <f aca="false">Inputs!$C$13/100*Inputs!$C$8</f>
         <v>0.6</v>
       </c>
-      <c r="N5" s="25" t="n">
+      <c r="N5" s="27" t="n">
         <f aca="false">M5-K5-L5-Inputs!$C$18</f>
         <v>0.24</v>
       </c>
-      <c r="O5" s="26" t="n">
+      <c r="O5" s="28" t="n">
         <f aca="false">N5*2*C5</f>
         <v>7.2</v>
       </c>
-      <c r="P5" s="26" t="n">
+      <c r="P5" s="28" t="n">
         <f aca="false">N5*F5*Inputs!$C$16+Inputs!$C$17</f>
         <v>10800</v>
       </c>
-      <c r="Q5" s="21" t="n">
+      <c r="Q5" s="23" t="n">
         <f aca="false">F5*Inputs!$C$16*Inputs!$C$14/100*Inputs!$C$11/1000</f>
         <v>35.775</v>
       </c>
-      <c r="R5" s="26" t="n">
+      <c r="R5" s="28" t="n">
         <f aca="false">IF(Q5&gt;0,P5/Q5,0)</f>
         <v>301.88679245283</v>
       </c>
-      <c r="S5" s="20" t="n">
+      <c r="S5" s="22" t="n">
         <f aca="false">J5*E5</f>
         <v>13500</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="B6" s="17" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="B6" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="C6" s="20" t="n">
         <v>160</v>
       </c>
-      <c r="D6" s="18" t="n">
+      <c r="D6" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="20" t="n">
+      <c r="F6" s="22" t="n">
         <f aca="false">2*C6*D6</f>
         <v>320</v>
       </c>
-      <c r="G6" s="21" t="n">
+      <c r="G6" s="23" t="n">
         <f aca="false">F6*Inputs!$C$13/100</f>
         <v>24</v>
       </c>
-      <c r="H6" s="22" t="n">
+      <c r="H6" s="24" t="n">
         <f aca="false">Inputs!$C$12*(1-Inputs!$C$15)</f>
         <v>26.775</v>
       </c>
-      <c r="I6" s="23" t="str">
+      <c r="I6" s="25" t="str">
         <f aca="false">IF(G6/D6&lt;=H6,"Yes","No – refuel at far end")</f>
         <v>Yes</v>
       </c>
-      <c r="J6" s="20" t="n">
+      <c r="J6" s="22" t="n">
         <f aca="false">G6*Inputs!$C$16</f>
         <v>6000</v>
       </c>
-      <c r="K6" s="24" t="n">
+      <c r="K6" s="26" t="n">
         <f aca="false">Inputs!$C$14/100*Inputs!$C$9</f>
         <v>0.36</v>
       </c>
-      <c r="L6" s="25" t="n">
+      <c r="L6" s="27" t="n">
         <f aca="false">Inputs!$C$14/100*Inputs!$C$11/1000*Inputs!$C$10</f>
         <v>0</v>
       </c>
-      <c r="M6" s="24" t="n">
+      <c r="M6" s="26" t="n">
         <f aca="false">Inputs!$C$13/100*Inputs!$C$8</f>
         <v>0.6</v>
       </c>
-      <c r="N6" s="25" t="n">
+      <c r="N6" s="27" t="n">
         <f aca="false">M6-K6-L6-Inputs!$C$18</f>
         <v>0.24</v>
       </c>
-      <c r="O6" s="26" t="n">
+      <c r="O6" s="28" t="n">
         <f aca="false">N6*2*C6</f>
         <v>76.8</v>
       </c>
-      <c r="P6" s="26" t="n">
+      <c r="P6" s="28" t="n">
         <f aca="false">N6*F6*Inputs!$C$16+Inputs!$C$17</f>
         <v>19200</v>
       </c>
-      <c r="Q6" s="21" t="n">
+      <c r="Q6" s="23" t="n">
         <f aca="false">F6*Inputs!$C$16*Inputs!$C$14/100*Inputs!$C$11/1000</f>
         <v>63.6</v>
       </c>
-      <c r="R6" s="26" t="n">
+      <c r="R6" s="28" t="n">
         <f aca="false">IF(Q6&gt;0,P6/Q6,0)</f>
         <v>301.88679245283</v>
       </c>
-      <c r="S6" s="20" t="n">
+      <c r="S6" s="22" t="n">
         <f aca="false">J6*E6</f>
         <v>18000</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="B7" s="17" t="s">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="B7" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="C7" s="20" t="n">
         <v>215</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="22" t="n">
         <f aca="false">2*C7*D7</f>
         <v>430</v>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="23" t="n">
         <f aca="false">F7*Inputs!$C$13/100</f>
         <v>32.25</v>
       </c>
-      <c r="H7" s="22" t="n">
+      <c r="H7" s="24" t="n">
         <f aca="false">Inputs!$C$12*(1-Inputs!$C$15)</f>
         <v>26.775</v>
       </c>
-      <c r="I7" s="23" t="str">
+      <c r="I7" s="25" t="str">
         <f aca="false">IF(G7/D7&lt;=H7,"Yes","No – refuel at far end")</f>
         <v>No – refuel at far end</v>
       </c>
-      <c r="J7" s="20" t="n">
+      <c r="J7" s="22" t="n">
         <f aca="false">G7*Inputs!$C$16</f>
         <v>8062.5</v>
       </c>
-      <c r="K7" s="24" t="n">
+      <c r="K7" s="26" t="n">
         <f aca="false">Inputs!$C$14/100*Inputs!$C$9</f>
         <v>0.36</v>
       </c>
-      <c r="L7" s="25" t="n">
+      <c r="L7" s="27" t="n">
         <f aca="false">Inputs!$C$14/100*Inputs!$C$11/1000*Inputs!$C$10</f>
         <v>0</v>
       </c>
-      <c r="M7" s="24" t="n">
+      <c r="M7" s="26" t="n">
         <f aca="false">Inputs!$C$13/100*Inputs!$C$8</f>
         <v>0.6</v>
       </c>
-      <c r="N7" s="25" t="n">
+      <c r="N7" s="27" t="n">
         <f aca="false">M7-K7-L7-Inputs!$C$18</f>
         <v>0.24</v>
       </c>
-      <c r="O7" s="26" t="n">
+      <c r="O7" s="28" t="n">
         <f aca="false">N7*2*C7</f>
         <v>103.2</v>
       </c>
-      <c r="P7" s="26" t="n">
+      <c r="P7" s="28" t="n">
         <f aca="false">N7*F7*Inputs!$C$16+Inputs!$C$17</f>
         <v>25800</v>
       </c>
-      <c r="Q7" s="21" t="n">
+      <c r="Q7" s="23" t="n">
         <f aca="false">F7*Inputs!$C$16*Inputs!$C$14/100*Inputs!$C$11/1000</f>
         <v>85.4625</v>
       </c>
-      <c r="R7" s="26" t="n">
+      <c r="R7" s="28" t="n">
         <f aca="false">IF(Q7&gt;0,P7/Q7,0)</f>
         <v>301.88679245283</v>
       </c>
-      <c r="S7" s="20" t="n">
+      <c r="S7" s="22" t="n">
         <f aca="false">J7*E7</f>
         <v>24187.5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="B8" s="17" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="B8" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="C8" s="20" t="n">
         <v>310</v>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F8" s="22" t="n">
         <f aca="false">2*C8*D8</f>
         <v>620</v>
       </c>
-      <c r="G8" s="21" t="n">
+      <c r="G8" s="23" t="n">
         <f aca="false">F8*Inputs!$C$13/100</f>
         <v>46.5</v>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="H8" s="24" t="n">
         <f aca="false">Inputs!$C$12*(1-Inputs!$C$15)</f>
         <v>26.775</v>
       </c>
-      <c r="I8" s="23" t="str">
+      <c r="I8" s="25" t="str">
         <f aca="false">IF(G8/D8&lt;=H8,"Yes","No – refuel at far end")</f>
         <v>No – refuel at far end</v>
       </c>
-      <c r="J8" s="20" t="n">
+      <c r="J8" s="22" t="n">
         <f aca="false">G8*Inputs!$C$16</f>
         <v>11625</v>
       </c>
-      <c r="K8" s="24" t="n">
+      <c r="K8" s="26" t="n">
         <f aca="false">Inputs!$C$14/100*Inputs!$C$9</f>
         <v>0.36</v>
       </c>
-      <c r="L8" s="25" t="n">
+      <c r="L8" s="27" t="n">
         <f aca="false">Inputs!$C$14/100*Inputs!$C$11/1000*Inputs!$C$10</f>
         <v>0</v>
       </c>
-      <c r="M8" s="24" t="n">
+      <c r="M8" s="26" t="n">
         <f aca="false">Inputs!$C$13/100*Inputs!$C$8</f>
         <v>0.6</v>
       </c>
-      <c r="N8" s="25" t="n">
+      <c r="N8" s="27" t="n">
         <f aca="false">M8-K8-L8-Inputs!$C$18</f>
         <v>0.24</v>
       </c>
-      <c r="O8" s="26" t="n">
+      <c r="O8" s="28" t="n">
         <f aca="false">N8*2*C8</f>
         <v>148.8</v>
       </c>
-      <c r="P8" s="26" t="n">
+      <c r="P8" s="28" t="n">
         <f aca="false">N8*F8*Inputs!$C$16+Inputs!$C$17</f>
         <v>37200</v>
       </c>
-      <c r="Q8" s="21" t="n">
+      <c r="Q8" s="23" t="n">
         <f aca="false">F8*Inputs!$C$16*Inputs!$C$14/100*Inputs!$C$11/1000</f>
         <v>123.225</v>
       </c>
-      <c r="R8" s="26" t="n">
+      <c r="R8" s="28" t="n">
         <f aca="false">IF(Q8&gt;0,P8/Q8,0)</f>
         <v>301.88679245283</v>
       </c>
-      <c r="S8" s="20" t="n">
+      <c r="S8" s="22" t="n">
         <f aca="false">J8*E8</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="B9" s="17" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="B9" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" s="20" t="n">
         <v>310</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="20" t="n">
+      <c r="F9" s="22" t="n">
         <f aca="false">2*C9*D9</f>
         <v>620</v>
       </c>
-      <c r="G9" s="21" t="n">
+      <c r="G9" s="23" t="n">
         <f aca="false">F9*Inputs!$C$13/100</f>
         <v>46.5</v>
       </c>
-      <c r="H9" s="22" t="n">
+      <c r="H9" s="24" t="n">
         <f aca="false">Inputs!$C$12*(1-Inputs!$C$15)</f>
         <v>26.775</v>
       </c>
-      <c r="I9" s="23" t="str">
+      <c r="I9" s="25" t="str">
         <f aca="false">IF(G9/D9&lt;=H9,"Yes","No – refuel at far end")</f>
         <v>No – refuel at far end</v>
       </c>
-      <c r="J9" s="20" t="n">
+      <c r="J9" s="22" t="n">
         <f aca="false">G9*Inputs!$C$16</f>
         <v>11625</v>
       </c>
-      <c r="K9" s="24" t="n">
+      <c r="K9" s="26" t="n">
         <f aca="false">Inputs!$C$14/100*Inputs!$C$9</f>
         <v>0.36</v>
       </c>
-      <c r="L9" s="25" t="n">
+      <c r="L9" s="27" t="n">
         <f aca="false">Inputs!$C$14/100*Inputs!$C$11/1000*Inputs!$C$10</f>
         <v>0</v>
       </c>
-      <c r="M9" s="24" t="n">
+      <c r="M9" s="26" t="n">
         <f aca="false">Inputs!$C$13/100*Inputs!$C$8</f>
         <v>0.6</v>
       </c>
-      <c r="N9" s="25" t="n">
+      <c r="N9" s="27" t="n">
         <f aca="false">M9-K9-L9-Inputs!$C$18</f>
         <v>0.24</v>
       </c>
-      <c r="O9" s="26" t="n">
+      <c r="O9" s="28" t="n">
         <f aca="false">N9*2*C9</f>
         <v>148.8</v>
       </c>
-      <c r="P9" s="26" t="n">
+      <c r="P9" s="28" t="n">
         <f aca="false">N9*F9*Inputs!$C$16+Inputs!$C$17</f>
         <v>37200</v>
       </c>
-      <c r="Q9" s="21" t="n">
+      <c r="Q9" s="23" t="n">
         <f aca="false">F9*Inputs!$C$16*Inputs!$C$14/100*Inputs!$C$11/1000</f>
         <v>123.225</v>
       </c>
-      <c r="R9" s="26" t="n">
+      <c r="R9" s="28" t="n">
         <f aca="false">IF(Q9&gt;0,P9/Q9,0)</f>
         <v>301.88679245283</v>
       </c>
-      <c r="S9" s="20" t="n">
+      <c r="S9" s="22" t="n">
         <f aca="false">J9*E9</f>
         <v>0</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="27" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="B10" s="19" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="C10" s="20" t="n">
+        <v>275</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <f aca="false">2*C10*D10</f>
+        <v>550</v>
+      </c>
+      <c r="G10" s="23" t="n">
+        <f aca="false">F10*Inputs!$C$13/100</f>
+        <v>41.25</v>
+      </c>
+      <c r="H10" s="24" t="n">
+        <f aca="false">Inputs!$C$12*(1-Inputs!$C$15)</f>
+        <v>26.775</v>
+      </c>
+      <c r="I10" s="25" t="str">
+        <f aca="false">IF(G10/D10&lt;=H10,"Yes","No – refuel at far end")</f>
+        <v>No – refuel at far end</v>
+      </c>
+      <c r="J10" s="22" t="n">
+        <f aca="false">G10*Inputs!$C$16</f>
+        <v>10312.5</v>
+      </c>
+      <c r="K10" s="26" t="n">
+        <f aca="false">Inputs!$C$14/100*Inputs!$C$9</f>
+        <v>0.36</v>
+      </c>
+      <c r="L10" s="27" t="n">
+        <f aca="false">Inputs!$C$14/100*Inputs!$C$11/1000*Inputs!$C$10</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="26" t="n">
+        <f aca="false">Inputs!$C$13/100*Inputs!$C$8</f>
+        <v>0.6</v>
+      </c>
+      <c r="N10" s="27" t="n">
+        <f aca="false">M10-K10-L10-Inputs!$C$18</f>
+        <v>0.24</v>
+      </c>
+      <c r="O10" s="28" t="n">
+        <f aca="false">N10*2*C10</f>
+        <v>132</v>
+      </c>
+      <c r="P10" s="28" t="n">
+        <f aca="false">N10*F10*Inputs!$C$16+Inputs!$C$17</f>
+        <v>33000</v>
+      </c>
+      <c r="Q10" s="23" t="n">
+        <f aca="false">F10*Inputs!$C$16*Inputs!$C$14/100*Inputs!$C$11/1000</f>
+        <v>109.3125</v>
+      </c>
+      <c r="R10" s="28" t="n">
+        <f aca="false">IF(Q10&gt;0,P10/Q10,0)</f>
+        <v>301.88679245283</v>
+      </c>
+      <c r="S10" s="22" t="n">
+        <f aca="false">J10*E10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="29"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="29" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>107</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="30" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="31" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -1965,208 +2282,208 @@
   <dimension ref="A1:C19"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="5" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="B5" s="28" t="n">
+      <c r="C4" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" s="32" t="n">
         <f aca="false">Inputs!$C$5</f>
         <v>127000</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="B6" s="29" t="n">
+      <c r="C5" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B6" s="33" t="n">
         <f aca="false">B5*Inputs!$C$7</f>
         <v>31750</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B7" s="30" t="n">
+      <c r="C6" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="34" t="n">
         <f aca="false">B5-B6</f>
         <v>95250</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="B8" s="29" t="n">
+      <c r="C7" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" s="33" t="n">
         <f aca="false">B7/Inputs!$C$16</f>
         <v>381</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="B9" s="28" t="n">
-        <f aca="false">SUM(Routes!S5:S9)</f>
+      <c r="C8" s="10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" s="32" t="n">
+        <f aca="false">SUM(Routes!S5:S10)</f>
         <v>55687.5</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="B10" s="31" t="n">
+      <c r="C9" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B10" s="35" t="n">
         <f aca="false">IF(B7&gt;0,B9/B7,0)</f>
         <v>0.584645669291339</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="B11" s="29" t="n">
+      <c r="C10" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" s="33" t="n">
         <f aca="false">B7-B9</f>
         <v>39562.5</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="B12" s="28" t="n">
-        <f aca="false">SUMPRODUCT(Routes!G5:G9,Routes!E5:E9)</f>
+      <c r="C11" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="B12" s="32" t="n">
+        <f aca="false">SUMPRODUCT(Routes!G5:G10,Routes!E5:E10)</f>
         <v>222.75</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="B13" s="6" t="str">
+      <c r="C12" s="10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B13" s="8" t="str">
         <f aca="false">IF(B12+B6/Inputs!$C$16&lt;=Inputs!$C$6,"Yes","No – add storage or stagger fills")</f>
         <v>Yes</v>
       </c>
-      <c r="C13" s="8"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="B14" s="28" t="n">
-        <f aca="false">SUM(Routes!E5:E9)</f>
+      <c r="C13" s="10"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B14" s="32" t="n">
+        <f aca="false">SUM(Routes!E5:E10)</f>
         <v>10</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="B15" s="32" t="n">
+      <c r="C14" s="10" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" s="36" t="n">
         <f aca="false">IF(Routes!J6&gt;0,B7/Routes!J6,0)</f>
         <v>15.875</v>
       </c>
-      <c r="C15" s="8" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="B16" s="33" t="n">
+      <c r="C15" s="10" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="B16" s="37" t="n">
         <f aca="false">B9*Inputs!$C$8</f>
         <v>445500</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="B17" s="34" t="n">
+      <c r="C16" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B17" s="38" t="n">
         <f aca="false">B7*Inputs!$C$8</f>
         <v>762000</v>
       </c>
-      <c r="C17" s="8" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="B18" s="32" t="n">
-        <f aca="false">SUMPRODUCT(Routes!Q5:Q9,Routes!E5:E9)</f>
+      <c r="C17" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B18" s="36" t="n">
+        <f aca="false">SUMPRODUCT(Routes!Q5:Q10,Routes!E5:E10)</f>
         <v>590.2875</v>
       </c>
-      <c r="C18" s="8" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="B19" s="35" t="n">
+      <c r="C18" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="B19" s="39" t="n">
         <f aca="false">Routes!S5+Routes!S6</f>
         <v>31500</v>
       </c>
-      <c r="C19" s="8" t="s">
-        <v>29</v>
+      <c r="C19" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -2185,321 +2502,519 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="58"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="40" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="31" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="41" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="41" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="41" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="43" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="45" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="42" t="s">
+        <v>138</v>
+      </c>
+      <c r="B6" s="46" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="44" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="45" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="42" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="46" t="n">
+        <v>12</v>
+      </c>
+      <c r="C7" s="44" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="45" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="42" t="s">
+        <v>142</v>
+      </c>
+      <c r="B8" s="47" t="n">
+        <f aca="false">B5*B6</f>
+        <v>12000</v>
+      </c>
+      <c r="C8" s="44" t="s">
+        <v>143</v>
+      </c>
+      <c r="D8" s="45"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="42" t="s">
+        <v>144</v>
+      </c>
+      <c r="B9" s="47" t="n">
+        <f aca="false">B5*B7</f>
+        <v>18000</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>143</v>
+      </c>
+      <c r="D9" s="45"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="B10" s="48" t="n">
+        <f aca="false">B5/Capacity!B7</f>
+        <v>0.015748031496063</v>
+      </c>
+      <c r="C10" s="44" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="45" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="42" t="s">
+        <v>147</v>
+      </c>
+      <c r="B11" s="49" t="n">
+        <f aca="false">B5/Capacity!B8</f>
+        <v>3.93700787401575</v>
+      </c>
+      <c r="C11" s="44" t="s">
+        <v>148</v>
+      </c>
+      <c r="D11" s="45" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="50" t="s">
+        <v>151</v>
+      </c>
+      <c r="B14" s="50" t="s">
+        <v>152</v>
+      </c>
+      <c r="C14" s="50" t="s">
+        <v>153</v>
+      </c>
+      <c r="D14" s="50" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="51" t="s">
+        <v>155</v>
+      </c>
+      <c r="B15" s="51" t="s">
+        <v>156</v>
+      </c>
+      <c r="C15" s="52" t="n">
+        <v>150</v>
+      </c>
+      <c r="D15" s="51" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="51" t="s">
+        <v>158</v>
+      </c>
+      <c r="B16" s="51" t="s">
+        <v>159</v>
+      </c>
+      <c r="C16" s="52" t="n">
+        <v>245</v>
+      </c>
+      <c r="D16" s="51" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="31" t="s">
+        <v>161</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F18"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>131</v>
-      </c>
-      <c r="B4" s="36" t="n">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="36" t="n">
+      <c r="C4" s="53" t="n">
         <v>45</v>
       </c>
-      <c r="D4" s="36" t="n">
+      <c r="D4" s="53" t="n">
         <v>70</v>
       </c>
-      <c r="E4" s="36" t="n">
+      <c r="E4" s="53" t="n">
         <v>100</v>
       </c>
-      <c r="F4" s="36" t="n">
+      <c r="F4" s="53" t="n">
         <v>200</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="37" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="54" t="n">
         <v>5</v>
       </c>
-      <c r="B5" s="38" t="n">
+      <c r="B5" s="55" t="n">
         <f aca="false">$A5*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*B$4)-Inputs!$C$18</f>
         <v>0.015</v>
       </c>
-      <c r="C5" s="38" t="n">
+      <c r="C5" s="55" t="n">
         <f aca="false">$A5*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*C$4)-Inputs!$C$18</f>
         <v>-0.020775</v>
       </c>
-      <c r="D5" s="38" t="n">
+      <c r="D5" s="55" t="n">
         <f aca="false">$A5*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*D$4)-Inputs!$C$18</f>
         <v>-0.04065</v>
       </c>
-      <c r="E5" s="38" t="n">
+      <c r="E5" s="55" t="n">
         <f aca="false">$A5*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*E$4)-Inputs!$C$18</f>
         <v>-0.0645</v>
       </c>
-      <c r="F5" s="38" t="n">
+      <c r="F5" s="55" t="n">
         <f aca="false">$A5*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*F$4)-Inputs!$C$18</f>
         <v>-0.144</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="37" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="54" t="n">
         <v>6</v>
       </c>
-      <c r="B6" s="38" t="n">
+      <c r="B6" s="55" t="n">
         <f aca="false">$A6*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*B$4)-Inputs!$C$18</f>
         <v>0.09</v>
       </c>
-      <c r="C6" s="38" t="n">
+      <c r="C6" s="55" t="n">
         <f aca="false">$A6*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*C$4)-Inputs!$C$18</f>
         <v>0.054225</v>
       </c>
-      <c r="D6" s="38" t="n">
+      <c r="D6" s="55" t="n">
         <f aca="false">$A6*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*D$4)-Inputs!$C$18</f>
         <v>0.0343500000000001</v>
       </c>
-      <c r="E6" s="38" t="n">
+      <c r="E6" s="55" t="n">
         <f aca="false">$A6*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*E$4)-Inputs!$C$18</f>
         <v>0.0105000000000001</v>
       </c>
-      <c r="F6" s="38" t="n">
+      <c r="F6" s="55" t="n">
         <f aca="false">$A6*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*F$4)-Inputs!$C$18</f>
         <v>-0.069</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="37" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="54" t="n">
         <v>7</v>
       </c>
-      <c r="B7" s="38" t="n">
+      <c r="B7" s="55" t="n">
         <f aca="false">$A7*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*B$4)-Inputs!$C$18</f>
         <v>0.165</v>
       </c>
-      <c r="C7" s="38" t="n">
+      <c r="C7" s="55" t="n">
         <f aca="false">$A7*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*C$4)-Inputs!$C$18</f>
         <v>0.129225</v>
       </c>
-      <c r="D7" s="38" t="n">
+      <c r="D7" s="55" t="n">
         <f aca="false">$A7*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*D$4)-Inputs!$C$18</f>
         <v>0.10935</v>
       </c>
-      <c r="E7" s="38" t="n">
+      <c r="E7" s="55" t="n">
         <f aca="false">$A7*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*E$4)-Inputs!$C$18</f>
         <v>0.0855000000000001</v>
       </c>
-      <c r="F7" s="38" t="n">
+      <c r="F7" s="55" t="n">
         <f aca="false">$A7*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*F$4)-Inputs!$C$18</f>
         <v>0.00600000000000001</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="37" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="54" t="n">
         <v>8</v>
       </c>
-      <c r="B8" s="38" t="n">
+      <c r="B8" s="55" t="n">
         <f aca="false">$A8*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*B$4)-Inputs!$C$18</f>
         <v>0.24</v>
       </c>
-      <c r="C8" s="38" t="n">
+      <c r="C8" s="55" t="n">
         <f aca="false">$A8*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*C$4)-Inputs!$C$18</f>
         <v>0.204225</v>
       </c>
-      <c r="D8" s="38" t="n">
+      <c r="D8" s="55" t="n">
         <f aca="false">$A8*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*D$4)-Inputs!$C$18</f>
         <v>0.18435</v>
       </c>
-      <c r="E8" s="38" t="n">
+      <c r="E8" s="55" t="n">
         <f aca="false">$A8*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*E$4)-Inputs!$C$18</f>
         <v>0.1605</v>
       </c>
-      <c r="F8" s="38" t="n">
+      <c r="F8" s="55" t="n">
         <f aca="false">$A8*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*F$4)-Inputs!$C$18</f>
         <v>0.081</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="37" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="54" t="n">
         <v>9</v>
       </c>
-      <c r="B9" s="38" t="n">
+      <c r="B9" s="55" t="n">
         <f aca="false">$A9*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*B$4)-Inputs!$C$18</f>
         <v>0.315</v>
       </c>
-      <c r="C9" s="38" t="n">
+      <c r="C9" s="55" t="n">
         <f aca="false">$A9*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*C$4)-Inputs!$C$18</f>
         <v>0.279225</v>
       </c>
-      <c r="D9" s="38" t="n">
+      <c r="D9" s="55" t="n">
         <f aca="false">$A9*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*D$4)-Inputs!$C$18</f>
         <v>0.25935</v>
       </c>
-      <c r="E9" s="38" t="n">
+      <c r="E9" s="55" t="n">
         <f aca="false">$A9*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*E$4)-Inputs!$C$18</f>
         <v>0.2355</v>
       </c>
-      <c r="F9" s="38" t="n">
+      <c r="F9" s="55" t="n">
         <f aca="false">$A9*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*F$4)-Inputs!$C$18</f>
         <v>0.156</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="37" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="54" t="n">
         <v>10</v>
       </c>
-      <c r="B10" s="38" t="n">
+      <c r="B10" s="55" t="n">
         <f aca="false">$A10*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*B$4)-Inputs!$C$18</f>
         <v>0.39</v>
       </c>
-      <c r="C10" s="38" t="n">
+      <c r="C10" s="55" t="n">
         <f aca="false">$A10*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*C$4)-Inputs!$C$18</f>
         <v>0.354225</v>
       </c>
-      <c r="D10" s="38" t="n">
+      <c r="D10" s="55" t="n">
         <f aca="false">$A10*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*D$4)-Inputs!$C$18</f>
         <v>0.33435</v>
       </c>
-      <c r="E10" s="38" t="n">
+      <c r="E10" s="55" t="n">
         <f aca="false">$A10*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*E$4)-Inputs!$C$18</f>
         <v>0.3105</v>
       </c>
-      <c r="F10" s="38" t="n">
+      <c r="F10" s="55" t="n">
         <f aca="false">$A10*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*F$4)-Inputs!$C$18</f>
         <v>0.231</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="37" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="54" t="n">
         <v>11</v>
       </c>
-      <c r="B11" s="38" t="n">
+      <c r="B11" s="55" t="n">
         <f aca="false">$A11*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*B$4)-Inputs!$C$18</f>
         <v>0.465</v>
       </c>
-      <c r="C11" s="38" t="n">
+      <c r="C11" s="55" t="n">
         <f aca="false">$A11*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*C$4)-Inputs!$C$18</f>
         <v>0.429225</v>
       </c>
-      <c r="D11" s="38" t="n">
+      <c r="D11" s="55" t="n">
         <f aca="false">$A11*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*D$4)-Inputs!$C$18</f>
         <v>0.40935</v>
       </c>
-      <c r="E11" s="38" t="n">
+      <c r="E11" s="55" t="n">
         <f aca="false">$A11*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*E$4)-Inputs!$C$18</f>
         <v>0.3855</v>
       </c>
-      <c r="F11" s="38" t="n">
+      <c r="F11" s="55" t="n">
         <f aca="false">$A11*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*F$4)-Inputs!$C$18</f>
         <v>0.306</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="54" t="n">
         <v>12</v>
       </c>
-      <c r="B12" s="38" t="n">
+      <c r="B12" s="55" t="n">
         <f aca="false">$A12*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*B$4)-Inputs!$C$18</f>
         <v>0.54</v>
       </c>
-      <c r="C12" s="38" t="n">
+      <c r="C12" s="55" t="n">
         <f aca="false">$A12*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*C$4)-Inputs!$C$18</f>
         <v>0.504225</v>
       </c>
-      <c r="D12" s="38" t="n">
+      <c r="D12" s="55" t="n">
         <f aca="false">$A12*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*D$4)-Inputs!$C$18</f>
         <v>0.48435</v>
       </c>
-      <c r="E12" s="38" t="n">
+      <c r="E12" s="55" t="n">
         <f aca="false">$A12*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*E$4)-Inputs!$C$18</f>
         <v>0.4605</v>
       </c>
-      <c r="F12" s="38" t="n">
+      <c r="F12" s="55" t="n">
         <f aca="false">$A12*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*F$4)-Inputs!$C$18</f>
         <v>0.381</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="37" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="54" t="n">
         <v>13</v>
       </c>
-      <c r="B13" s="38" t="n">
+      <c r="B13" s="55" t="n">
         <f aca="false">$A13*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*B$4)-Inputs!$C$18</f>
         <v>0.615</v>
       </c>
-      <c r="C13" s="38" t="n">
+      <c r="C13" s="55" t="n">
         <f aca="false">$A13*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*C$4)-Inputs!$C$18</f>
         <v>0.579225</v>
       </c>
-      <c r="D13" s="38" t="n">
+      <c r="D13" s="55" t="n">
         <f aca="false">$A13*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*D$4)-Inputs!$C$18</f>
         <v>0.55935</v>
       </c>
-      <c r="E13" s="38" t="n">
+      <c r="E13" s="55" t="n">
         <f aca="false">$A13*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*E$4)-Inputs!$C$18</f>
         <v>0.5355</v>
       </c>
-      <c r="F13" s="38" t="n">
+      <c r="F13" s="55" t="n">
         <f aca="false">$A13*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*F$4)-Inputs!$C$18</f>
         <v>0.456</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="37" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="54" t="n">
         <v>14</v>
       </c>
-      <c r="B14" s="38" t="n">
+      <c r="B14" s="55" t="n">
         <f aca="false">$A14*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*B$4)-Inputs!$C$18</f>
         <v>0.69</v>
       </c>
-      <c r="C14" s="38" t="n">
+      <c r="C14" s="55" t="n">
         <f aca="false">$A14*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*C$4)-Inputs!$C$18</f>
         <v>0.654225</v>
       </c>
-      <c r="D14" s="38" t="n">
+      <c r="D14" s="55" t="n">
         <f aca="false">$A14*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*D$4)-Inputs!$C$18</f>
         <v>0.63435</v>
       </c>
-      <c r="E14" s="38" t="n">
+      <c r="E14" s="55" t="n">
         <f aca="false">$A14*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*E$4)-Inputs!$C$18</f>
         <v>0.6105</v>
       </c>
-      <c r="F14" s="38" t="n">
+      <c r="F14" s="55" t="n">
         <f aca="false">$A14*Inputs!$C$13/100-Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*F$4)-Inputs!$C$18</f>
         <v>0.531</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="B16" s="39" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="B16" s="56" t="n">
         <f aca="false">(Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*B$4)+Inputs!$C$18)/(Inputs!$C$13/100)</f>
         <v>4.8</v>
       </c>
-      <c r="C16" s="39" t="n">
+      <c r="C16" s="56" t="n">
         <f aca="false">(Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*C$4)+Inputs!$C$18)/(Inputs!$C$13/100)</f>
         <v>5.277</v>
       </c>
-      <c r="D16" s="39" t="n">
+      <c r="D16" s="56" t="n">
         <f aca="false">(Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*D$4)+Inputs!$C$18)/(Inputs!$C$13/100)</f>
         <v>5.542</v>
       </c>
-      <c r="E16" s="39" t="n">
+      <c r="E16" s="56" t="n">
         <f aca="false">(Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*E$4)+Inputs!$C$18)/(Inputs!$C$13/100)</f>
         <v>5.86</v>
       </c>
-      <c r="F16" s="39" t="n">
+      <c r="F16" s="56" t="n">
         <f aca="false">(Inputs!$C$14/100*(Inputs!$C$9+Inputs!$C$11/1000*F$4)+Inputs!$C$18)/(Inputs!$C$13/100)</f>
         <v>6.92</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>133</v>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>